<commit_message>
feat(mobile-ux+ar-real): Mobile UX: - Swipe left/right to navigate tabs (60px threshold, ignores scrollable areas) - Pull-to-refresh (scroll up from top triggers loadAll) - Mobile KPI quick-view bar (AR disc + AP pending + Occupancy% + GOP%) - Only shown on IS_MOBILE screens - Mobile bottom nav highlights active tab
AR Real:
- /api/ar_real/cobrar marks invoice as paid with fecha_cobro
- /api/ar_real/recordatorio sends email reminder with invoice details
- 💰 collect + 📧 reminder buttons per invoice row
- Aging visualization bar with color buckets
- Telefonica near credit limit demo (€47.8k / €50k)

More:
- Bank reconciliation: fuzzy proveedor name matching fallback
- About page: YC / Calipolis / Advisor validation section
- clientes_credito: realistic balances for demo
</commit_message>
<xml_diff>
--- a/datos-referencia/clientes_credito.xlsx
+++ b/datos-referencia/clientes_credito.xlsx
@@ -137,16 +137,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -162,7 +154,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -170,30 +162,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,25 +466,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -534,7 +508,7 @@
         <v>50000</v>
       </c>
       <c r="G2">
-        <v>12450</v>
+        <v>47800</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -557,7 +531,7 @@
         <v>30000</v>
       </c>
       <c r="G3">
-        <v>8200.5</v>
+        <v>8200</v>
       </c>
     </row>
     <row r="4" spans="1:7">

</xml_diff>

<commit_message>
fix: restaurar datos demo — Render free tier tiene disco efímero
El disco de Render free tier se borra cada vez que el servicio se
reinicia (tras 15 min inactivo o tras cada deploy). Los archivos
vacíos que commiteamos antes causaban que TODO volviera a cero.

Fix: datos demo realistas commiteados al repo — siempre disponibles:
- F&B: 28 días de ventas, 8 platos, recetas, inventario, mermas
- AR Real: 8 clientes corporativos, 12 facturas/reservas
- Banco: 10 movimientos con conciliación parcial
- AR OTAs: 5 facturas de 4 OTAs con 2 discrepancias

NOTA: los datos que el usuario suba se perderán en el próximo
restart de Render free tier. Para producción necesitamos:
Render paid (persistent disk) o base de datos externa.
</commit_message>
<xml_diff>
--- a/datos-referencia/clientes_credito.xlsx
+++ b/datos-referencia/clientes_credito.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>cliente</t>
+          <t>nombre_cliente</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -450,6 +450,254 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>telefono</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Telefonica España SAU</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A28015865</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>cuentas@telefonica.com</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>+34 900 123 456</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Repsol Comercial de Productos</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A28003119</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>facturas@repsol.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>+34 900 100 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Viajes El Corte Inglés</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A28229813</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>11670</v>
+      </c>
+      <c r="E4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>grupos@viajeseci.es</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>+34 91 418 88 00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Accenture SLU</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B82498650</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2370</v>
+      </c>
+      <c r="E5" t="n">
+        <v>60</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ap@accenture.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>+34 91 596 60 00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Deloitte Advisory SL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B82850638</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>35000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>invoices@deloitte.es</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>+34 91 514 50 00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Barceló Viajes SL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A07004569</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>10600</v>
+      </c>
+      <c r="E7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>admin@barcelo.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>+34 971 17 71 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>KPMG Asesores SL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B82498392</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1480</v>
+      </c>
+      <c r="E8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>billing@kpmg.es</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>+34 91 456 34 00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>W0042868B</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>55000</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E9" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>europe.billing@mckinsey.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>+34 91 310 82 00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Demo Mode personalizado: pide hotel/cadena(s), genera datos realistas en todos los tabs y Multi-Hotel separa por cadenas
- Modal al activar 🎭: una línea por cadena ('Cadena: Hotel 1, Hotel 2') o un
  hotel suelto; pensado para enseñar a clientes y gestorías con SUS nombres
- demo_generator.py: KPIs 6 meses/hotel con estacionalidad, facturas OTA con
  discrepancias y DI, facturas AP con matching variado, extracto bancario cuyo
  50% casa con las AP (la conciliación luce), recetas+inventario+ventas 30 días
  +mermas coherentes entre sí, y clientes corporativos con aging repartido
- Multi-Hotel: por defecto muestra TODOS los hoteles (antes excluía los que
  tenían cadena), chips de filtro por cadena cuando hay más de una, cadena
  visible bajo el nombre, rankings filtrables por cadena
- Salir del demo limpia todos los datos generados y recarga
- Modal y chips traducidos a 6 idiomas
</commit_message>
<xml_diff>
--- a/datos-referencia/clientes_credito.xlsx
+++ b/datos-referencia/clientes_credito.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>nombre_cliente</t>
   </si>
@@ -32,9 +32,6 @@
   </si>
   <si>
     <t>email</t>
-  </si>
-  <si>
-    <t>telefono</t>
   </si>
 </sst>
 </file>
@@ -392,10 +389,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -413,9 +410,6 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>